<commit_message>
update and new files
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,19 +511,19 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>44556.57706018518</v>
+        <v>44561.058125</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>26.12.2021</t>
+          <t>31.12.2021</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>*7197</t>
+          <t>*5091</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-600</v>
+        <v>-564</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>-600</v>
+        <v>-564</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -550,87 +550,25 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Цветы</t>
+          <t>Различные товары</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>5992</v>
+        <v>5399</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>IP Isaeva O.N.</t>
+          <t>Ozon.ru</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>198</v>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>44527.62321759259</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>27.11.2021</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>*7197</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>-500</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>-500</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>RUB</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Цветы</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
-        <v>5992</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>IP Isaeva O.N.</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>10</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>500</v>
+        <v>564</v>
       </c>
     </row>
   </sheetData>

</xml_diff>